<commit_message>
Mise à jour du code
</commit_message>
<xml_diff>
--- a/cotisations.xlsx
+++ b/cotisations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\cotisation_streamlit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6471AB7C-F558-4F84-A36D-373A0D28F58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44BE1DE7-52B6-43F1-BA45-F9B10A5A2696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D47798F2-2E3F-4123-AE53-AE0EE02E72EF}"/>
   </bookViews>
@@ -3372,7 +3372,7 @@
         <v>16</v>
       </c>
       <c r="D205" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.35">
@@ -4226,7 +4226,7 @@
         <v>5</v>
       </c>
       <c r="D266" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Modification du fichier excel
</commit_message>
<xml_diff>
--- a/cotisations.xlsx
+++ b/cotisations.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\cotisation_streamlit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\cotisations_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08515B92-CD4A-4647-A107-763BCAFAEF2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D13297A-C587-41DE-ADC2-D053BC462176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D47798F2-2E3F-4123-AE53-AE0EE02E72EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$D$290</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3022,7 +3025,7 @@
         <v>15</v>
       </c>
       <c r="D180" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.35">
@@ -3036,7 +3039,7 @@
         <v>16</v>
       </c>
       <c r="D181" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.35">
@@ -3162,7 +3165,7 @@
         <v>13</v>
       </c>
       <c r="D190" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.35">
@@ -3176,7 +3179,7 @@
         <v>14</v>
       </c>
       <c r="D191" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.35">
@@ -3190,7 +3193,7 @@
         <v>15</v>
       </c>
       <c r="D192" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.35">
@@ -3204,7 +3207,7 @@
         <v>16</v>
       </c>
       <c r="D193" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.35">
@@ -3358,7 +3361,7 @@
         <v>15</v>
       </c>
       <c r="D204" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.35">
@@ -3372,7 +3375,7 @@
         <v>16</v>
       </c>
       <c r="D205" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.35">
@@ -3442,7 +3445,7 @@
         <v>9</v>
       </c>
       <c r="D210" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.35">
@@ -3456,7 +3459,7 @@
         <v>10</v>
       </c>
       <c r="D211" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.35">
@@ -3470,7 +3473,7 @@
         <v>11</v>
       </c>
       <c r="D212" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.35">
@@ -3484,7 +3487,7 @@
         <v>12</v>
       </c>
       <c r="D213" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.35">
@@ -3498,7 +3501,7 @@
         <v>13</v>
       </c>
       <c r="D214" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
@@ -3512,7 +3515,7 @@
         <v>14</v>
       </c>
       <c r="D215" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
@@ -3526,7 +3529,7 @@
         <v>15</v>
       </c>
       <c r="D216" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.35">
@@ -3540,7 +3543,7 @@
         <v>16</v>
       </c>
       <c r="D217" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
@@ -3554,7 +3557,7 @@
         <v>5</v>
       </c>
       <c r="D218" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.35">
@@ -3568,7 +3571,7 @@
         <v>6</v>
       </c>
       <c r="D219" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.35">
@@ -3890,7 +3893,7 @@
         <v>5</v>
       </c>
       <c r="D242" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.35">
@@ -4058,7 +4061,7 @@
         <v>5</v>
       </c>
       <c r="D254" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.35">
@@ -4072,7 +4075,7 @@
         <v>6</v>
       </c>
       <c r="D255" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.35">
@@ -4086,7 +4089,7 @@
         <v>7</v>
       </c>
       <c r="D256" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.35">
@@ -4100,7 +4103,7 @@
         <v>8</v>
       </c>
       <c r="D257" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.35">
@@ -4114,7 +4117,7 @@
         <v>9</v>
       </c>
       <c r="D258" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.35">
@@ -4128,7 +4131,7 @@
         <v>10</v>
       </c>
       <c r="D259" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.35">
@@ -4226,7 +4229,7 @@
         <v>5</v>
       </c>
       <c r="D266" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.35">
@@ -4394,7 +4397,7 @@
         <v>5</v>
       </c>
       <c r="D278" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.35">
@@ -4408,7 +4411,7 @@
         <v>6</v>
       </c>
       <c r="D279" s="3">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.35">
@@ -4564,6 +4567,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D290" xr:uid="{77FEF14F-85DA-4ECB-B2FA-74F479AC4B4A}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>